<commit_message>
Agregar formato visual al Excel y dashboard HTML ejecutivo
- Excel: tablas nativas, encabezados azules, colores ABC/riesgo/pedido,
  semáforo por celda, resumen ejecutivo destacado
- Dashboard HTML para audiencia no técnica: KPIs, acciones, top 5,
  gráfico de ventas y modelos a producir
- Módulos excel_format.py y dashboard_html.py integrados al script principal

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analisis_microfibra_jabon.xlsx
+++ b/analisis_microfibra_jabon.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,16 +37,94 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,12 +132,72 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4C6E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -134,6 +272,169 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_1ResumenporColor" displayName="T_1ResumenporColor" ref="A1:W24" headerRowCount="1">
+  <autoFilter ref="A1:W24"/>
+  <tableColumns count="23">
+    <tableColumn id="1" name="Color"/>
+    <tableColumn id="2" name="ABC"/>
+    <tableColumn id="3" name="Ventas 10m (u)"/>
+    <tableColumn id="4" name="% Total"/>
+    <tableColumn id="5" name="Venta prom (u/mes)"/>
+    <tableColumn id="6" name="CV mensual"/>
+    <tableColumn id="7" name="Modelos"/>
+    <tableColumn id="8" name="Géneros"/>
+    <tableColumn id="9" name="Inv PT (u)"/>
+    <tableColumn id="10" name="Cob. PT (meses)"/>
+    <tableColumn id="11" name="Tela actual (kg)"/>
+    <tableColumn id="12" name="Consumo kg/mes"/>
+    <tableColumn id="13" name="kg/u pond."/>
+    <tableColumn id="14" name="Cob. tela (meses)"/>
+    <tableColumn id="15" name="Riesgo"/>
+    <tableColumn id="16" name="Acción sugerida"/>
+    <tableColumn id="17" name="Venta proy. horizonte (u)"/>
+    <tableColumn id="18" name="Prod. requerida (u)"/>
+    <tableColumn id="19" name="Kg prod. c/merma"/>
+    <tableColumn id="20" name="SS tela (kg)"/>
+    <tableColumn id="21" name="Necesidad neta (kg)"/>
+    <tableColumn id="22" name="Pedido sugerido (kg)"/>
+    <tableColumn id="23" name="Cob. tela post-pedido (meses)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_2Top5Logística" displayName="T_2Top5Logística" ref="A1:O6" headerRowCount="1">
+  <autoFilter ref="A1:O6"/>
+  <tableColumns count="15">
+    <tableColumn id="1" name="Top 5 Logística"/>
+    <tableColumn id="2" name="Color"/>
+    <tableColumn id="3" name="Ventas 10m (u)"/>
+    <tableColumn id="4" name="% Total"/>
+    <tableColumn id="5" name="Venta prom (u/mes)"/>
+    <tableColumn id="6" name="CV mensual"/>
+    <tableColumn id="7" name="Modelos"/>
+    <tableColumn id="8" name="Géneros"/>
+    <tableColumn id="9" name="Cobertura PT (meses)"/>
+    <tableColumn id="10" name="Score rotación (40%)"/>
+    <tableColumn id="11" name="Score regularidad (25%)"/>
+    <tableColumn id="12" name="Score transversal (20%)"/>
+    <tableColumn id="13" name="Score no-inmov (15%)"/>
+    <tableColumn id="14" name="SCORE TOTAL"/>
+    <tableColumn id="15" name="Justificación"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_3RiesgoyReorden" displayName="T_3RiesgoyReorden" ref="A1:W17" headerRowCount="1">
+  <autoFilter ref="A1:W17"/>
+  <tableColumns count="23">
+    <tableColumn id="1" name="Color"/>
+    <tableColumn id="2" name="ABC"/>
+    <tableColumn id="3" name="Ventas 10m (u)"/>
+    <tableColumn id="4" name="% Total"/>
+    <tableColumn id="5" name="Venta prom (u/mes)"/>
+    <tableColumn id="6" name="CV mensual"/>
+    <tableColumn id="7" name="Modelos"/>
+    <tableColumn id="8" name="Géneros"/>
+    <tableColumn id="9" name="Inv PT (u)"/>
+    <tableColumn id="10" name="Cob. PT (meses)"/>
+    <tableColumn id="11" name="Tela actual (kg)"/>
+    <tableColumn id="12" name="Consumo kg/mes"/>
+    <tableColumn id="13" name="kg/u pond."/>
+    <tableColumn id="14" name="Cob. tela (meses)"/>
+    <tableColumn id="15" name="Riesgo"/>
+    <tableColumn id="16" name="Acción sugerida"/>
+    <tableColumn id="17" name="Venta proy. horizonte (u)"/>
+    <tableColumn id="18" name="Prod. requerida (u)"/>
+    <tableColumn id="19" name="Kg prod. c/merma"/>
+    <tableColumn id="20" name="SS tela (kg)"/>
+    <tableColumn id="21" name="Necesidad neta (kg)"/>
+    <tableColumn id="22" name="Pedido sugerido (kg)"/>
+    <tableColumn id="23" name="Cob. tela post-pedido (meses)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T_4PedidoTela" displayName="T_4PedidoTela" ref="A1:I4" headerRowCount="1">
+  <autoFilter ref="A1:I4"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Color"/>
+    <tableColumn id="2" name="ABC"/>
+    <tableColumn id="3" name="Tela actual (kg)"/>
+    <tableColumn id="4" name="Consumo kg/mes"/>
+    <tableColumn id="5" name="Prod. requerida (u)"/>
+    <tableColumn id="6" name="Necesidad neta (kg)"/>
+    <tableColumn id="7" name="Pedido sugerido (kg)"/>
+    <tableColumn id="8" name="Cob. tela post-pedido (meses)"/>
+    <tableColumn id="9" name="Acción sugerida"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T_5ResumenModelos" displayName="T_5ResumenModelos" ref="A1:G21" headerRowCount="1">
+  <autoFilter ref="A1:G21"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Modelo"/>
+    <tableColumn id="2" name="Ventas 10m"/>
+    <tableColumn id="3" name="Venta prom/mes"/>
+    <tableColumn id="4" name="Inv PT"/>
+    <tableColumn id="5" name="Cob. PT (meses)"/>
+    <tableColumn id="6" name="Venta proy."/>
+    <tableColumn id="7" name="Prod. requerida"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_10SemáforoIntegrado" displayName="T_10SemáforoIntegrado" ref="A1:N24" headerRowCount="1">
+  <autoFilter ref="A1:N24"/>
+  <tableColumns count="14">
+    <tableColumn id="1" name="Color"/>
+    <tableColumn id="2" name="ABC"/>
+    <tableColumn id="3" name="Venta prom (u/mes)"/>
+    <tableColumn id="4" name="% Total"/>
+    <tableColumn id="5" name="CV mensual"/>
+    <tableColumn id="6" name="Cob. PT (meses)"/>
+    <tableColumn id="7" name="Cob. tela (meses)"/>
+    <tableColumn id="8" name="Rotación"/>
+    <tableColumn id="9" name="Regularidad"/>
+    <tableColumn id="10" name="Riesgo PT"/>
+    <tableColumn id="11" name="Riesgo Tela"/>
+    <tableColumn id="12" name="Prod. requerida (u)"/>
+    <tableColumn id="13" name="Pedido tela (kg)"/>
+    <tableColumn id="14" name="Acción integrada"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_11VerificaciónyNotas" displayName="T_11VerificaciónyNotas" ref="A1:I24" headerRowCount="1">
+  <autoFilter ref="A1:I24"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Color"/>
+    <tableColumn id="2" name="Consumo kg/mes"/>
+    <tableColumn id="3" name="kg/u pond."/>
+    <tableColumn id="4" name="Cob. tela (meses)"/>
+    <tableColumn id="5" name="Prod. requerida (u)"/>
+    <tableColumn id="6" name="Pedido sugerido (kg)"/>
+    <tableColumn id="7" name="Riesgo"/>
+    <tableColumn id="8" name="Acción sugerida"/>
+    <tableColumn id="9" name="Notas verificación"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -427,16 +728,15 @@
   </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Valor</t>
         </is>
       </c>
     </row>
@@ -446,149 +746,151 @@
           <t>PLANIFICACIÓN TELA JABÓN MICROFIBRA — RESUMEN EJECUTIVO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Ventas analizadas</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>26,427 u en 10 meses · 20 productos · 23 colores</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Inventario PT actual</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>21,202 u ≈ 8.0 meses</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Tela jabón en almacén MP</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>4,157.9 kg en 13 colores</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Lead time tela</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>45 días (1.5 meses)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Horizonte pedido</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Ago-Dic 2026 · MEQ = 5.88 meses</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Pedido tela sugerido (total)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>390 kg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Producción PT requerida (total)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2,507 u</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Top 5 Logística (rotación + bajo riesgo inmov.)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Negro, Blanco, Azul Marino, Azul Lavanda, Verde Militar</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Crítico operativo (pedido tela)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Lila, Rojo, Púrpura</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Metodología pedido</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Prod = Venta proy + Stock PT obj (1.5m) − Inv PT · Tela = kg prod × 1.05 + SS(z×σ×√LT) − Inv tela</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Supuestos</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Nov 1.20× · Dic 1.96× · tienda +10% desde oct · merma 5% · pedido min 50 kg</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1831,74 +2133,90 @@
   </sheetPr>
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Venta prom (u/mes)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>% Total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>CV mensual</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Cob. PT (meses)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela (meses)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Rotación</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Regularidad</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Riesgo PT</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Riesgo Tela</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida (u)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Pedido tela (kg)</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Acción integrada</t>
         </is>
@@ -1930,7 +2248,7 @@
       <c r="G2" t="n">
         <v>2.680804138201173</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1940,12 +2258,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="17" t="inlineStr">
         <is>
           <t>CRÍTICO</t>
         </is>
@@ -1988,22 +2306,22 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2046,22 +2364,22 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>SOBRESTOCK</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2104,22 +2422,22 @@
       <c r="G5" t="n">
         <v>4.93853641839169</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2162,22 +2480,22 @@
       <c r="G6" t="n">
         <v>2.365058701024037</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t>CRÍTICO</t>
         </is>
@@ -2220,22 +2538,22 @@
       <c r="G7" t="n">
         <v>5.886532347553176</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2278,22 +2596,22 @@
       <c r="G8" t="n">
         <v>3.956420485611875</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>BAJO</t>
         </is>
@@ -2336,22 +2654,22 @@
       <c r="G9" t="n">
         <v>5.940664164340741</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2394,22 +2712,22 @@
       <c r="G10" t="n">
         <v>1.581946787387088</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>CRÍTICO</t>
         </is>
@@ -2452,22 +2770,22 @@
       <c r="G11" t="n">
         <v>3.552696511215744</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="18" t="inlineStr">
         <is>
           <t>SOBRESTOCK</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="18" t="inlineStr">
         <is>
           <t>BAJO</t>
         </is>
@@ -2510,22 +2828,22 @@
       <c r="G12" t="n">
         <v>6.185435163076219</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="18" t="inlineStr">
         <is>
           <t>SOBRESTOCK</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2568,22 +2886,22 @@
       <c r="G13" t="n">
         <v>3.636231331091616</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="18" t="inlineStr">
         <is>
           <t>BAJO</t>
         </is>
@@ -2631,17 +2949,17 @@
           <t>BAJA</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="18" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="18" t="inlineStr">
         <is>
           <t>SOBRESTOCK</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="17" t="inlineStr">
         <is>
           <t>CRÍTICO</t>
         </is>
@@ -2689,17 +3007,17 @@
           <t>BAJA</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="18" t="inlineStr">
         <is>
           <t>SOBRESTOCK</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>CRÍTICO</t>
         </is>
@@ -2752,12 +3070,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2810,12 +3128,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2868,12 +3186,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2926,12 +3244,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -2984,12 +3302,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -3042,12 +3360,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -3100,12 +3418,12 @@
           <t>MODA/PIco</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -3153,17 +3471,17 @@
           <t>BAJA</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -3211,17 +3529,17 @@
           <t>BAJA</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
         <is>
           <t>QUIEBRE</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" s="17" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -3240,6 +3558,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3251,49 +3572,60 @@
   </sheetPr>
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Consumo kg/mes</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>kg/u pond.</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela (meses)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida (u)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Pedido sugerido (kg)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Riesgo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Acción sugerida</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Notas verificación</t>
         </is>
@@ -4152,6 +4484,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -4163,119 +4498,144 @@
   </sheetPr>
   <dimension ref="A1:W24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="31" customWidth="1" min="23" max="23"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ventas 10m (u)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>% Total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Venta prom (u/mes)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>CV mensual</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Modelos</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Géneros</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Inv PT (u)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Cob. PT (meses)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Tela actual (kg)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Consumo kg/mes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>kg/u pond.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela (meses)</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Riesgo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Acción sugerida</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>Venta proy. horizonte (u)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida (u)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>Kg prod. c/merma</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>SS tela (kg)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>Necesidad neta (kg)</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>Pedido sugerido (kg)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela post-pedido (meses)</t>
         </is>
@@ -4287,7 +4647,7 @@
           <t>Negro</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4328,7 +4688,7 @@
       <c r="N2" t="n">
         <v>3.956420485611875</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="8" t="inlineStr">
         <is>
           <t>SALUDABLE</t>
         </is>
@@ -4366,7 +4726,7 @@
           <t>Blanco</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4407,7 +4767,7 @@
       <c r="N3" t="n">
         <v>5.886532347553176</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>SALUDABLE</t>
         </is>
@@ -4445,7 +4805,7 @@
           <t>Azul Marino</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4486,7 +4846,7 @@
       <c r="N4" t="n">
         <v>4.93853641839169</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>SALUDABLE</t>
         </is>
@@ -4524,7 +4884,7 @@
           <t>Lila</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4565,7 +4925,7 @@
       <c r="N5" t="n">
         <v>2.680804138201173</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -4603,7 +4963,7 @@
           <t>Azul Lavanda</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4644,7 +5004,7 @@
       <c r="N6" t="n">
         <v>2.365058701024037</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -4682,7 +5042,7 @@
           <t>Verde Militar</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4723,7 +5083,7 @@
       <c r="N7" t="n">
         <v>1.581946787387088</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -4761,7 +5121,7 @@
           <t>Azul Rey</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4802,7 +5162,7 @@
       <c r="N8" t="n">
         <v>5.940664164340741</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="8" t="inlineStr">
         <is>
           <t>SALUDABLE</t>
         </is>
@@ -4840,7 +5200,7 @@
           <t>Aguamarina</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4881,7 +5241,7 @@
       <c r="N9" t="n">
         <v>6.185435163076219</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="10" t="inlineStr">
         <is>
           <t>SOBRE-STOCK PT</t>
         </is>
@@ -4919,7 +5279,7 @@
           <t>Rojo</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -4960,7 +5320,7 @@
       <c r="N10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -4998,7 +5358,7 @@
           <t>Vinotinto</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -5039,7 +5399,7 @@
       <c r="N11" t="n">
         <v>3.552696511215744</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="10" t="inlineStr">
         <is>
           <t>SOBRE-STOCK PT</t>
         </is>
@@ -5077,7 +5437,7 @@
           <t>Gris Claro</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -5118,7 +5478,7 @@
       <c r="N12" t="n">
         <v>3.636231331091616</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>SALUDABLE</t>
         </is>
@@ -5156,7 +5516,7 @@
           <t>Púrpura</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -5197,7 +5557,7 @@
       <c r="N13" t="n">
         <v>0</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -5235,7 +5595,7 @@
           <t>Rosado Pastel</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -5276,7 +5636,7 @@
       <c r="N14" t="n">
         <v>1.443237121218717</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5314,7 +5674,7 @@
           <t>Amarillo Neón</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5355,7 +5715,7 @@
       <c r="N15" t="n">
         <v>2.469051073018744</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5393,7 +5753,7 @@
           <t>Azul Cielo</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5434,7 +5794,7 @@
       <c r="N16" t="n">
         <v>0</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5472,7 +5832,7 @@
           <t>Rosado Neón</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5513,7 +5873,7 @@
       <c r="N17" t="n">
         <v>0</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5551,7 +5911,7 @@
           <t>Morado</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5592,7 +5952,7 @@
       <c r="N18" t="n">
         <v>0</v>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O18" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5630,7 +5990,7 @@
           <t>Azul Turquesa</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5671,7 +6031,7 @@
       <c r="N19" t="n">
         <v>0</v>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O19" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5709,7 +6069,7 @@
           <t>Amarillo Pastel</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5750,7 +6110,7 @@
       <c r="N20" t="n">
         <v>0</v>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5788,7 +6148,7 @@
           <t>Fucsia</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5829,7 +6189,7 @@
       <c r="N21" t="n">
         <v>24.37182213433382</v>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>QUIEBRE PT</t>
         </is>
@@ -5867,7 +6227,7 @@
           <t>Coral Neón</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5908,7 +6268,7 @@
       <c r="N22" t="n">
         <v>0</v>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -5946,7 +6306,7 @@
           <t>Morado Uva</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -5987,7 +6347,7 @@
       <c r="N23" t="n">
         <v>0</v>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -6025,7 +6385,7 @@
           <t>Gris Oscuro</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -6066,7 +6426,7 @@
       <c r="N24" t="n">
         <v>0</v>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O24" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -6100,6 +6460,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -6111,79 +6474,96 @@
   </sheetPr>
   <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Top 5 Logística</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ventas 10m (u)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>% Total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Venta prom (u/mes)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>CV mensual</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Modelos</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Géneros</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Cobertura PT (meses)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Score rotación (40%)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Score regularidad (25%)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Score transversal (20%)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Score no-inmov (15%)</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>SCORE TOTAL</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Justificación</t>
         </is>
@@ -6231,7 +6611,7 @@
       <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="13" t="n">
         <v>94.2</v>
       </c>
       <c r="O2" t="inlineStr">
@@ -6282,7 +6662,7 @@
       <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="13" t="n">
         <v>87.2</v>
       </c>
       <c r="O3" t="inlineStr">
@@ -6333,7 +6713,7 @@
       <c r="M4" t="n">
         <v>100</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="13" t="n">
         <v>81.40000000000001</v>
       </c>
       <c r="O4" t="inlineStr">
@@ -6384,7 +6764,7 @@
       <c r="M5" t="n">
         <v>100</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="13" t="n">
         <v>68.40000000000001</v>
       </c>
       <c r="O5" t="inlineStr">
@@ -6435,7 +6815,7 @@
       <c r="M6" t="n">
         <v>70</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="13" t="n">
         <v>65.7</v>
       </c>
       <c r="O6" t="inlineStr">
@@ -6446,6 +6826,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -6457,119 +6840,144 @@
   </sheetPr>
   <dimension ref="A1:W17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="31" customWidth="1" min="23" max="23"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ventas 10m (u)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>% Total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Venta prom (u/mes)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>CV mensual</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Modelos</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Géneros</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Inv PT (u)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Cob. PT (meses)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Tela actual (kg)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Consumo kg/mes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>kg/u pond.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela (meses)</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Riesgo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Acción sugerida</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>Venta proy. horizonte (u)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida (u)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>Kg prod. c/merma</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>SS tela (kg)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>Necesidad neta (kg)</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>Pedido sugerido (kg)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela post-pedido (meses)</t>
         </is>
@@ -6622,7 +7030,7 @@
       <c r="N2" t="n">
         <v>2.680804138201173</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -6701,7 +7109,7 @@
       <c r="N3" t="n">
         <v>2.365058701024037</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -6780,7 +7188,7 @@
       <c r="N4" t="n">
         <v>1.581946787387088</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -6859,7 +7267,7 @@
       <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -6938,7 +7346,7 @@
       <c r="N6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>SIN TELA</t>
         </is>
@@ -7017,7 +7425,7 @@
       <c r="N7" t="n">
         <v>1.443237121218717</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7096,7 +7504,7 @@
       <c r="N8" t="n">
         <v>2.469051073018744</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7175,7 +7583,7 @@
       <c r="N9" t="n">
         <v>0</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7254,7 +7662,7 @@
       <c r="N10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7333,7 +7741,7 @@
       <c r="N11" t="n">
         <v>0</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7412,7 +7820,7 @@
       <c r="N12" t="n">
         <v>0</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7491,7 +7899,7 @@
       <c r="N13" t="n">
         <v>0</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7570,7 +7978,7 @@
       <c r="N14" t="n">
         <v>24.37182213433382</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>QUIEBRE PT</t>
         </is>
@@ -7649,7 +8057,7 @@
       <c r="N15" t="n">
         <v>0</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7728,7 +8136,7 @@
       <c r="N16" t="n">
         <v>0</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7807,7 +8215,7 @@
       <c r="N17" t="n">
         <v>0</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>TELA CRÍTICA</t>
         </is>
@@ -7841,6 +8249,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -7852,154 +8263,165 @@
   </sheetPr>
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Tela actual (kg)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Consumo kg/mes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida (u)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Necesidad neta (kg)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Pedido sugerido (kg)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Cob. tela post-pedido (meses)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Acción sugerida</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Lila</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="14" t="n">
         <v>188.44</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="14" t="n">
         <v>70.29234150856085</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="14" t="n">
         <v>731.8362500000001</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="14" t="n">
         <v>285.592117585966</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="15" t="n">
         <v>290</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="14" t="n">
         <v>6.806431393976698</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="14" t="inlineStr">
         <is>
           <t>Incluir en pedido o priorizar consumo</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Rojo</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="C3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="14" t="n">
         <v>52.36383642495785</v>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="E3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="14" t="n">
         <v>43.53188649067186</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="14" t="n">
         <v>0.954857462967874</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>Incluir en pedido — sin capacidad de reacción</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Púrpura</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="C4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="14" t="n">
         <v>32.06584398976982</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="E4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14" t="n">
         <v>20.95965792154968</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="14" t="n">
         <v>1.559291563195774</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>Incluir en pedido — sin capacidad de reacción</t>
         </is>
@@ -8007,6 +8429,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -8018,39 +8443,48 @@
   </sheetPr>
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Ventas 10m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Venta prom/mes</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Inv PT</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Cob. PT (meses)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Venta proy.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Prod. requerida</t>
         </is>
@@ -8558,6 +8992,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>